<commit_message>
Deploy the implementation guide.
</commit_message>
<xml_diff>
--- a/docs/CodeSystem-bioinfo-analysis-code.xlsx
+++ b/docs/CodeSystem-bioinfo-analysis-code.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="48">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-01-22T16:34:58+00:00</t>
+    <t>2026-02-20T16:31:02+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -123,7 +123,7 @@
     <t>Count</t>
   </si>
   <si>
-    <t>5</t>
+    <t>3</t>
   </si>
   <si>
     <t>Level</t>
@@ -141,34 +141,22 @@
     <t>1</t>
   </si>
   <si>
-    <t>RABA</t>
-  </si>
-  <si>
-    <t>Reads Alignement Bioinformatic Analysis</t>
-  </si>
-  <si>
-    <t>SNVC</t>
-  </si>
-  <si>
-    <t>SNV Calling Bioinformatic Analysis</t>
-  </si>
-  <si>
-    <t>QCBA</t>
-  </si>
-  <si>
-    <t>Quality Control Bioinformatic Analysis</t>
-  </si>
-  <si>
-    <t>GEBA</t>
-  </si>
-  <si>
-    <t>Germline Exome Bioinformatic Analysis</t>
-  </si>
-  <si>
-    <t>GGBA</t>
-  </si>
-  <si>
-    <t>Germline Genome Bioinformatic Analysis</t>
+    <t>GBVA</t>
+  </si>
+  <si>
+    <t>Germline Variant Analysis</t>
+  </si>
+  <si>
+    <t>GBVF</t>
+  </si>
+  <si>
+    <t>Germline Variant Analysis with Family Joint Genotyping</t>
+  </si>
+  <si>
+    <t>SBVA</t>
+  </si>
+  <si>
+    <t>Somatic Variant Analysis</t>
   </si>
 </sst>
 </file>
@@ -478,7 +466,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -531,30 +519,6 @@
       </c>
       <c r="D4" s="2"/>
     </row>
-    <row r="5">
-      <c r="A5" t="s" s="2">
-        <v>41</v>
-      </c>
-      <c r="B5" t="s" s="2">
-        <v>48</v>
-      </c>
-      <c r="C5" t="s" s="2">
-        <v>49</v>
-      </c>
-      <c r="D5" s="2"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="s" s="2">
-        <v>41</v>
-      </c>
-      <c r="B6" t="s" s="2">
-        <v>50</v>
-      </c>
-      <c r="C6" t="s" s="2">
-        <v>51</v>
-      </c>
-      <c r="D6" s="2"/>
-    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>